<commit_message>
Costo de tokens: recalibrado con los cinco tableros medidos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01163dWk83hFd4E5njufh21p
</commit_message>
<xml_diff>
--- a/AUREA_Costo_Tokens_IC.xlsx
+++ b/AUREA_Costo_Tokens_IC.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Precios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Cuadro" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Medido en esta sesión" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tableros medidos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -80,6 +81,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -607,7 +611,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tokens y costo por canal y tamaño de base · estimación en sesión nueva con el kit AUREA (±30%)</t>
+          <t>Tokens y costo por canal y tamaño de base · recalibrado con los 5 tableros medidos (DRAKON, TKVA, PAVIR, EDFAN, BETROX) · sesión nueva con el kit · ±30%</t>
         </is>
       </c>
     </row>
@@ -701,7 +705,7 @@
         <v>110</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>300</v>
+        <v>675</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>55</v>
@@ -748,13 +752,13 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>130</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>80</v>
@@ -807,7 +811,7 @@
         <v>150</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>550</v>
+        <v>1238</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>110</v>
@@ -860,7 +864,7 @@
         <v>100</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>220</v>
+        <v>495</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>40</v>
@@ -913,7 +917,7 @@
         <v>110</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>280</v>
+        <v>630</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>55</v>
@@ -966,7 +970,7 @@
         <v>125</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>380</v>
+        <v>855</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>75</v>
@@ -1019,7 +1023,7 @@
         <v>100</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>220</v>
+        <v>495</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>40</v>
@@ -1072,7 +1076,7 @@
         <v>115</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>300</v>
+        <v>675</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>55</v>
@@ -1125,7 +1129,7 @@
         <v>130</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>75</v>
@@ -1178,7 +1182,7 @@
         <v>95</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>180</v>
+        <v>405</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>35</v>
@@ -1231,7 +1235,7 @@
         <v>105</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>230</v>
+        <v>518</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>45</v>
@@ -1284,7 +1288,7 @@
         <v>115</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>300</v>
+        <v>675</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>60</v>
@@ -1337,7 +1341,7 @@
         <v>95</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>180</v>
+        <v>405</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>35</v>
@@ -1390,7 +1394,7 @@
         <v>105</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>220</v>
+        <v>495</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>45</v>
@@ -1443,7 +1447,7 @@
         <v>115</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>290</v>
+        <v>652</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>60</v>
@@ -1496,7 +1500,7 @@
         <v>95</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>180</v>
+        <v>405</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>35</v>
@@ -1549,7 +1553,7 @@
         <v>105</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>230</v>
+        <v>518</v>
       </c>
       <c r="G20" s="5" t="n">
         <v>45</v>
@@ -1602,7 +1606,7 @@
         <v>115</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>300</v>
+        <v>675</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>60</v>
@@ -1655,7 +1659,7 @@
         <v>140</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>200</v>
+        <v>450</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>40</v>
@@ -1708,7 +1712,7 @@
         <v>170</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>300</v>
+        <v>675</v>
       </c>
       <c r="G23" s="5" t="n">
         <v>60</v>
@@ -1761,7 +1765,7 @@
         <v>200</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>80</v>
@@ -1895,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2056,6 +2060,336 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Corrección: el primer cálculo (USD 16,70) incluía por error los primeros pasos del cálculo de tokens. El tablero BETROX solo: 25,8 M tokens · USD 14,42.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Tablero</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Base que usó</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Pestañas</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Rondas de cambios</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Pasos</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Tokens (M)</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>Contexto medio por paso (miles)</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>USD a precio Opus 5.5</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>USD real (modelo que se usó en ese momento)</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DRAKON</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ilustrativo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Quincena: 74 mensajes, USD 271 mil de pauta, Meta + Google + Calor de muestra</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Diseño + 2 rondas de Sofi</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>152</v>
+      </c>
+      <c r="G2" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>446</v>
+      </c>
+      <c r="I2" t="n">
+        <v>32.23</v>
+      </c>
+      <c r="J2" t="n">
+        <v>54.31</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Opus 4.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TKVA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1.113 contactos × 30 columnas</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G3" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>391</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Opus 4.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PAVIR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ilustrativo</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4.950 consultas/mes, 700 distribuidores, pedidos, deuda, Meta, Google, email, WhatsApp</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Base + 2 ampliaciones + ajustes</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>311</v>
+      </c>
+      <c r="G4" t="n">
+        <v>111.6</v>
+      </c>
+      <c r="H4" t="n">
+        <v>350</v>
+      </c>
+      <c r="I4" t="n">
+        <v>50.08</v>
+      </c>
+      <c r="J4" t="n">
+        <v>89.79000000000001</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Opus 4.8 y Opus 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EDFAN Real Estate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.017 contactos × 41 columnas</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tablero + curaduría completa</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>93</v>
+      </c>
+      <c r="G5" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="H5" t="n">
+        <v>415</v>
+      </c>
+      <c r="I5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="J5" t="n">
+        <v>32.04</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Opus 4.8 y Opus 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BETROX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>942 contactos × 43 columnas</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1 (primera vez)</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>59</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>420</v>
+      </c>
+      <c r="I6" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="J6" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fuera de los tableros: skills de curaduría USD 10,66 · export MD USD 2,00 · reporte de metodologías USD 5,77 · kit USD 15,32 (precio Opus 5.5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lectura: en datos reales el costo lo mueve la curaduría (columnas, cruces, insights). En los ilustrativos lo movieron las rondas de diseño y la cantidad de pestañas, no el volumen de datos.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Costo de tokens: la actualización queda como columna de uso normal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01163dWk83hFd4E5njufh21p
</commit_message>
<xml_diff>
--- a/AUREA_Costo_Tokens_IC.xlsx
+++ b/AUREA_Costo_Tokens_IC.xlsx
@@ -615,6 +615,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Uso normal: columna ACTUALIZACIÓN. El tablero ya existe y se regenera con cada export nuevo. El ALTA se paga una sola vez por cliente o por canal nuevo.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -653,27 +660,27 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Tokens · primera vez</t>
+          <t>Tokens · alta (cliente o canal nuevo, una sola vez)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>USD Opus · primera vez</t>
+          <t>USD Opus · alta (una sola vez)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Tokens · actualización</t>
+          <t>Tokens · actualización con export nuevo (estructura ya hecha)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>USD Opus · actualización</t>
+          <t>USD Opus · actualización (cada export)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>USD Sonnet · actualización</t>
+          <t>USD Sonnet · actualización (cada export)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Costo de tokens: Grande recalibrado a escala PAVIR/DRAKON + columna de margen de precio
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01163dWk83hFd4E5njufh21p
</commit_message>
<xml_diff>
--- a/AUREA_Costo_Tokens_IC.xlsx
+++ b/AUREA_Costo_Tokens_IC.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -38,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +56,11 @@
         <fgColor rgb="00EEF0FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D5B"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -83,6 +89,10 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -577,6 +587,26 @@
       </c>
       <c r="B11" s="5" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Margen de precio sugerido (multiplicador sobre el costo de API)</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Margen de precio sugerido 2 (escenario conservador)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -590,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -606,19 +636,22 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tokens y costo por canal y tamaño de base · recalibrado con los 5 tableros medidos (DRAKON, TKVA, PAVIR, EDFAN, BETROX) · sesión nueva con el kit · ±30%</t>
+          <t>Tokens y costo por canal y tamaño de base · Grande = escala real PAVIR/DRAKON (sesiones separadas por canal) · ±30%</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Uso normal: columna ACTUALIZACIÓN. El tablero ya existe y se regenera con cada export nuevo. El ALTA se paga una sola vez por cliente o por canal nuevo.</t>
+          <t>Chica/Mediana ancladas a lo medido (TKVA, BETROX, EDFAN). Grande es ~2x la Mediana real, consistente con que PAVIR/DRAKON (un tablero grande armado en una sola sesión) salió USD 32-50: armar cada canal en sesiones separadas cuesta más por no compartir caché entre canales.</t>
         </is>
       </c>
     </row>
@@ -688,6 +721,21 @@
           <t>ARS Opus · actualización</t>
         </is>
       </c>
+      <c r="N3" s="12" t="inlineStr">
+        <is>
+          <t>Precio sugerido · alta (2,5x)</t>
+        </is>
+      </c>
+      <c r="O3" s="12" t="inlineStr">
+        <is>
+          <t>Precio sugerido · actualización (2,5x)</t>
+        </is>
+      </c>
+      <c r="P3" s="12" t="inlineStr">
+        <is>
+          <t>Precio sugerido · actualización (4x, conservador)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -712,10 +760,10 @@
         <v>110</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>675</v>
+        <v>776</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="H4" s="6">
         <f>(D4*E4+F4+G4)*1000</f>
@@ -741,6 +789,18 @@
         <f>K4*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N4" s="7">
+        <f>I4*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O4" s="7">
+        <f>K4*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P4" s="7">
+        <f>K4*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -759,16 +819,16 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>900</v>
+        <v>1395</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>80</v>
+        <v>124</v>
       </c>
       <c r="H5" s="6">
         <f>(D5*E5+F5+G5)*1000</f>
@@ -794,6 +854,18 @@
         <f>K5*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N5" s="7">
+        <f>I5*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O5" s="7">
+        <f>K5*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P5" s="7">
+        <f>K5*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -812,16 +884,16 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>150</v>
+        <v>172</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1238</v>
+        <v>3033</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>110</v>
+        <v>270</v>
       </c>
       <c r="H6" s="6">
         <f>(D6*E6+F6+G6)*1000</f>
@@ -847,6 +919,18 @@
         <f>K6*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N6" s="7">
+        <f>I6*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O6" s="7">
+        <f>K6*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P6" s="7">
+        <f>K6*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -871,10 +955,10 @@
         <v>100</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>495</v>
+        <v>569</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H7" s="6">
         <f>(D7*E7+F7+G7)*1000</f>
@@ -900,6 +984,18 @@
         <f>K7*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N7" s="7">
+        <f>I7*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O7" s="7">
+        <f>K7*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P7" s="7">
+        <f>K7*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -918,16 +1014,16 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>630</v>
+        <v>976</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="H8" s="6">
         <f>(D8*E8+F8+G8)*1000</f>
@@ -953,6 +1049,18 @@
         <f>K8*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N8" s="7">
+        <f>I8*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O8" s="7">
+        <f>K8*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P8" s="7">
+        <f>K8*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -971,16 +1079,16 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>855</v>
+        <v>2095</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>75</v>
+        <v>184</v>
       </c>
       <c r="H9" s="6">
         <f>(D9*E9+F9+G9)*1000</f>
@@ -1006,6 +1114,18 @@
         <f>K9*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N9" s="7">
+        <f>I9*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O9" s="7">
+        <f>K9*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P9" s="7">
+        <f>K9*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1030,10 +1150,10 @@
         <v>100</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>495</v>
+        <v>569</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H10" s="6">
         <f>(D10*E10+F10+G10)*1000</f>
@@ -1059,6 +1179,18 @@
         <f>K10*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N10" s="7">
+        <f>I10*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O10" s="7">
+        <f>K10*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P10" s="7">
+        <f>K10*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1077,16 +1209,16 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>675</v>
+        <v>1046</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="H11" s="6">
         <f>(D11*E11+F11+G11)*1000</f>
@@ -1112,6 +1244,18 @@
         <f>K11*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N11" s="7">
+        <f>I11*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O11" s="7">
+        <f>K11*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P11" s="7">
+        <f>K11*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1130,16 +1274,16 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>900</v>
+        <v>2205</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>75</v>
+        <v>184</v>
       </c>
       <c r="H12" s="6">
         <f>(D12*E12+F12+G12)*1000</f>
@@ -1165,6 +1309,18 @@
         <f>K12*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N12" s="7">
+        <f>I12*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O12" s="7">
+        <f>K12*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P12" s="7">
+        <f>K12*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1189,10 +1345,10 @@
         <v>95</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>405</v>
+        <v>466</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H13" s="6">
         <f>(D13*E13+F13+G13)*1000</f>
@@ -1218,6 +1374,18 @@
         <f>K13*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N13" s="7">
+        <f>I13*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O13" s="7">
+        <f>K13*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P13" s="7">
+        <f>K13*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1236,16 +1404,16 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>518</v>
+        <v>803</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="H14" s="6">
         <f>(D14*E14+F14+G14)*1000</f>
@@ -1271,6 +1439,18 @@
         <f>K14*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N14" s="7">
+        <f>I14*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O14" s="7">
+        <f>K14*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P14" s="7">
+        <f>K14*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1289,16 +1469,16 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>675</v>
+        <v>1654</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>60</v>
+        <v>147</v>
       </c>
       <c r="H15" s="6">
         <f>(D15*E15+F15+G15)*1000</f>
@@ -1324,6 +1504,18 @@
         <f>K15*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N15" s="7">
+        <f>I15*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O15" s="7">
+        <f>K15*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P15" s="7">
+        <f>K15*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1348,10 +1540,10 @@
         <v>95</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>405</v>
+        <v>466</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H16" s="6">
         <f>(D16*E16+F16+G16)*1000</f>
@@ -1377,6 +1569,18 @@
         <f>K16*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N16" s="7">
+        <f>I16*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O16" s="7">
+        <f>K16*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P16" s="7">
+        <f>K16*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1395,16 +1599,16 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>495</v>
+        <v>767</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="H17" s="6">
         <f>(D17*E17+F17+G17)*1000</f>
@@ -1430,6 +1634,18 @@
         <f>K17*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N17" s="7">
+        <f>I17*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O17" s="7">
+        <f>K17*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P17" s="7">
+        <f>K17*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1448,16 +1664,16 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>652</v>
+        <v>1597</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>60</v>
+        <v>147</v>
       </c>
       <c r="H18" s="6">
         <f>(D18*E18+F18+G18)*1000</f>
@@ -1483,6 +1699,18 @@
         <f>K18*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N18" s="7">
+        <f>I18*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O18" s="7">
+        <f>K18*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P18" s="7">
+        <f>K18*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1507,10 +1735,10 @@
         <v>95</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>405</v>
+        <v>466</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H19" s="6">
         <f>(D19*E19+F19+G19)*1000</f>
@@ -1536,6 +1764,18 @@
         <f>K19*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N19" s="7">
+        <f>I19*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O19" s="7">
+        <f>K19*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P19" s="7">
+        <f>K19*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1554,16 +1794,16 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>518</v>
+        <v>803</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="H20" s="6">
         <f>(D20*E20+F20+G20)*1000</f>
@@ -1589,6 +1829,18 @@
         <f>K20*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N20" s="7">
+        <f>I20*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O20" s="7">
+        <f>K20*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P20" s="7">
+        <f>K20*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1607,16 +1859,16 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>675</v>
+        <v>1654</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>60</v>
+        <v>147</v>
       </c>
       <c r="H21" s="6">
         <f>(D21*E21+F21+G21)*1000</f>
@@ -1642,6 +1894,18 @@
         <f>K21*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N21" s="7">
+        <f>I21*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O21" s="7">
+        <f>K21*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P21" s="7">
+        <f>K21*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1666,10 +1930,10 @@
         <v>140</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>450</v>
+        <v>518</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H22" s="6">
         <f>(D22*E22+F22+G22)*1000</f>
@@ -1695,6 +1959,18 @@
         <f>K22*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N22" s="7">
+        <f>I22*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O22" s="7">
+        <f>K22*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P22" s="7">
+        <f>K22*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1713,16 +1989,16 @@
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>675</v>
+        <v>1046</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="H23" s="6">
         <f>(D23*E23+F23+G23)*1000</f>
@@ -1748,6 +2024,18 @@
         <f>K23*Precios!$B$11</f>
         <v/>
       </c>
+      <c r="N23" s="7">
+        <f>I23*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O23" s="7">
+        <f>K23*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P23" s="7">
+        <f>K23*Precios!$B$14</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1766,16 +2054,16 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>900</v>
+        <v>2205</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>80</v>
+        <v>196</v>
       </c>
       <c r="H24" s="6">
         <f>(D24*E24+F24+G24)*1000</f>
@@ -1801,7 +2089,20 @@
         <f>K24*Precios!$B$11</f>
         <v/>
       </c>
-    </row>
+      <c r="N24" s="7">
+        <f>I24*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O24" s="7">
+        <f>K24*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P24" s="7">
+        <f>K24*Precios!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
@@ -1832,6 +2133,18 @@
         <f>SUMIF($B$4:$B$24,"Chica",M$4:M$24)</f>
         <v/>
       </c>
+      <c r="N26">
+        <f>SUMIF($B$4:$B$24,"Chica",N$4:N$24)</f>
+        <v/>
+      </c>
+      <c r="O26">
+        <f>SUMIF($B$4:$B$24,"Chica",O$4:O$24)</f>
+        <v/>
+      </c>
+      <c r="P26">
+        <f>SUMIF($B$4:$B$24,"Chica",P$4:P$24)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -1863,6 +2176,18 @@
         <f>SUMIF($B$4:$B$24,"Mediana",M$4:M$24)</f>
         <v/>
       </c>
+      <c r="N27">
+        <f>SUMIF($B$4:$B$24,"Mediana",N$4:N$24)</f>
+        <v/>
+      </c>
+      <c r="O27">
+        <f>SUMIF($B$4:$B$24,"Mediana",O$4:O$24)</f>
+        <v/>
+      </c>
+      <c r="P27">
+        <f>SUMIF($B$4:$B$24,"Mediana",P$4:P$24)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -1894,7 +2219,20 @@
         <f>SUMIF($B$4:$B$24,"Grande",M$4:M$24)</f>
         <v/>
       </c>
-    </row>
+      <c r="N28">
+        <f>SUMIF($B$4:$B$24,"Grande",N$4:N$24)</f>
+        <v/>
+      </c>
+      <c r="O28">
+        <f>SUMIF($B$4:$B$24,"Grande",O$4:O$24)</f>
+        <v/>
+      </c>
+      <c r="P28">
+        <f>SUMIF($B$4:$B$24,"Grande",P$4:P$24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Costo de tokens: escenario optimizado sin pérdida de calidad
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01163dWk83hFd4E5njufh21p
</commit_message>
<xml_diff>
--- a/AUREA_Costo_Tokens_IC.xlsx
+++ b/AUREA_Costo_Tokens_IC.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Cuadro" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Medido en esta sesión" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tableros medidos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Escenario optimizado" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -93,6 +94,9 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -620,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2102,7 +2106,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
@@ -2232,7 +2235,6 @@
         <v/>
       </c>
     </row>
-    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2738,4 +2740,789 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Costo por actualización (USD, Opus 5.5) aplicando mejoras que no sacrifican calidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Paso 1: sesión nueva por export, sin compactación, y verificación con el verificador automático + 2 capturas (contexto nuevo escrito −36%). Paso 2: además, una sola sesión por cliente con todos los canales (caché compartido, −30%). Paso 3: además, pipeline propio por API con caché de 5 minutos (escritura USD 5 en vez de 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Canal</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Tamaño</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Hoy (cuadro)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Paso 1</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Paso 2</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Paso 3</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Precio 2,5x sobre Paso 2</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Precio 4x sobre Paso 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Prometheo (CRM)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>7.56</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Prometheo (CRM)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>14.21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prometheo (CRM)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>14.71</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>30.18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>5.46</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>9.460000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>20.18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>5.46</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>10.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>21.13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LinkedIn Ads</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LinkedIn Ads</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>7.75</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LinkedIn Ads</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>15.84</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WhatsApp Marketing</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WhatsApp Marketing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>7.52</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WhatsApp Marketing</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Email Marketing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Email Marketing</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>7.78</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Email Marketing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>15.87</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cruce omnicanal</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Chica</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>5.21</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cruce omnicanal</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>10.57</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cruce omnicanal</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>5.52</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>22.06</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Tablero completo · Chica</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>23.23</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>37.17</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Tablero completo · Mediana</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>32.91</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>24.05</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>16.83</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>67.34</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Tablero completo · Grande</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>68.95999999999999</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>50.24</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>35.17</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>26.43</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>87.92</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>140.67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Documento de costo de IC: Opus, Opus + Sonnet, mejoras y harness
Recalibrado con el costo en sesión nueva de los cinco tableros,
derivado llamada por llamada del registro real. La planilla anterior
queda marcada como desactualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01163dWk83hFd4E5njufh21p
</commit_message>
<xml_diff>
--- a/AUREA_Costo_Tokens_IC.xlsx
+++ b/AUREA_Costo_Tokens_IC.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
     </font>
   </fonts>
   <fills count="5">
@@ -75,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -98,6 +102,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -624,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -646,164 +651,106 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>DESACTUALIZADO: estos valores se calibraron con costos inflados por la conversación larga. La versión vigente es AUREA_Costo_IC.html (costos en sesión nueva, medidos llamada por llamada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Tokens y costo por canal y tamaño de base · Grande = escala real PAVIR/DRAKON (sesiones separadas por canal) · ±30%</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Chica/Mediana ancladas a lo medido (TKVA, BETROX, EDFAN). Grande es ~2x la Mediana real, consistente con que PAVIR/DRAKON (un tablero grande armado en una sola sesión) salió USD 32-50: armar cada canal en sesiones separadas cuesta más por no compartir caché entre canales.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Canal</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Tamaño</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Qué significa el tamaño</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Pasos (llamadas)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Contexto medio por paso (miles)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Contexto nuevo escrito (miles)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Salida (miles)</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Tokens · alta (cliente o canal nuevo, una sola vez)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>USD Opus · alta (una sola vez)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Tokens · actualización con export nuevo (estructura ya hecha)</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>USD Opus · actualización (cada export)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>USD Sonnet · actualización (cada export)</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>ARS Opus · actualización</t>
         </is>
       </c>
-      <c r="N3" s="12" t="inlineStr">
+      <c r="N4" s="12" t="inlineStr">
         <is>
           <t>Precio sugerido · alta (2,5x)</t>
         </is>
       </c>
-      <c r="O3" s="12" t="inlineStr">
+      <c r="O4" s="12" t="inlineStr">
         <is>
           <t>Precio sugerido · actualización (2,5x)</t>
         </is>
       </c>
-      <c r="P3" s="12" t="inlineStr">
+      <c r="P4" s="12" t="inlineStr">
         <is>
           <t>Precio sugerido · actualización (4x, conservador)</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Prometheo (CRM)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Chica</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>hasta 300 contactos, ~25 columnas</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>110</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>776</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="H4" s="6">
-        <f>(D4*E4+F4+G4)*1000</f>
-        <v/>
-      </c>
-      <c r="I4" s="7">
-        <f>(D4*E4*Precios!$B$4+F4*Precios!$B$5+G4*Precios!$B$6)/1000</f>
-        <v/>
-      </c>
-      <c r="J4" s="6">
-        <f>H4*Precios!$B$10</f>
-        <v/>
-      </c>
-      <c r="K4" s="7">
-        <f>I4*Precios!$B$10</f>
-        <v/>
-      </c>
-      <c r="L4" s="7">
-        <f>(D4*E4*Precios!$C$4+F4*Precios!$C$5+G4*Precios!$C$6)/1000*Precios!$B$10</f>
-        <v/>
-      </c>
-      <c r="M4" s="6">
-        <f>K4*Precios!$B$11</f>
-        <v/>
-      </c>
-      <c r="N4" s="7">
-        <f>I4*Precios!$B$13</f>
-        <v/>
-      </c>
-      <c r="O4" s="7">
-        <f>K4*Precios!$B$13</f>
-        <v/>
-      </c>
-      <c r="P4" s="7">
-        <f>K4*Precios!$B$14</f>
-        <v/>
       </c>
     </row>
     <row r="5">
@@ -814,60 +761,60 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>~1.000 contactos, ~40 columnas (BETROX, EDFAN)</t>
+          <t>hasta 300 contactos, ~25 columnas</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1395</v>
+        <v>776</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>124</v>
+        <v>63</v>
       </c>
       <c r="H5" s="6">
-        <f>(D5*E5+F5+G5)*1000</f>
+        <f>(D4*E4+F4+G4)*1000</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>(D5*E5*Precios!$B$4+F5*Precios!$B$5+G5*Precios!$B$6)/1000</f>
+        <f>(D4*E4*Precios!$B$4+F4*Precios!$B$5+G4*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J5" s="6">
-        <f>H5*Precios!$B$10</f>
+        <f>H4*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K5" s="7">
-        <f>I5*Precios!$B$10</f>
+        <f>I4*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L5" s="7">
-        <f>(D5*E5*Precios!$C$4+F5*Precios!$C$5+G5*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D4*E4*Precios!$C$4+F4*Precios!$C$5+G4*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M5" s="6">
-        <f>K5*Precios!$B$11</f>
+        <f>K4*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N5" s="7">
-        <f>I5*Precios!$B$13</f>
+        <f>I4*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O5" s="7">
-        <f>K5*Precios!$B$13</f>
+        <f>K4*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P5" s="7">
-        <f>K5*Precios!$B$14</f>
+        <f>K4*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -879,125 +826,125 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.000+ contactos, 50+ columnas, varios embudos</t>
+          <t>~1.000 contactos, ~40 columnas (BETROX, EDFAN)</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>3033</v>
+        <v>1395</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>270</v>
+        <v>124</v>
       </c>
       <c r="H6" s="6">
-        <f>(D6*E6+F6+G6)*1000</f>
+        <f>(D5*E5+F5+G5)*1000</f>
         <v/>
       </c>
       <c r="I6" s="7">
-        <f>(D6*E6*Precios!$B$4+F6*Precios!$B$5+G6*Precios!$B$6)/1000</f>
+        <f>(D5*E5*Precios!$B$4+F5*Precios!$B$5+G5*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J6" s="6">
-        <f>H6*Precios!$B$10</f>
+        <f>H5*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K6" s="7">
-        <f>I6*Precios!$B$10</f>
+        <f>I5*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L6" s="7">
-        <f>(D6*E6*Precios!$C$4+F6*Precios!$C$5+G6*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D5*E5*Precios!$C$4+F5*Precios!$C$5+G5*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M6" s="6">
-        <f>K6*Precios!$B$11</f>
+        <f>K5*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>I6*Precios!$B$13</f>
+        <f>I5*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O6" s="7">
-        <f>K6*Precios!$B$13</f>
+        <f>K5*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P6" s="7">
-        <f>K6*Precios!$B$14</f>
+        <f>K5*Precios!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Prometheo (CRM)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>hasta 10 anuncios, 1 mes</t>
+          <t>5.000+ contactos, 50+ columnas, varios embudos</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>100</v>
+        <v>172</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>569</v>
+        <v>3033</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>46</v>
+        <v>270</v>
       </c>
       <c r="H7" s="6">
-        <f>(D7*E7+F7+G7)*1000</f>
+        <f>(D6*E6+F6+G6)*1000</f>
         <v/>
       </c>
       <c r="I7" s="7">
-        <f>(D7*E7*Precios!$B$4+F7*Precios!$B$5+G7*Precios!$B$6)/1000</f>
+        <f>(D6*E6*Precios!$B$4+F6*Precios!$B$5+G6*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J7" s="6">
-        <f>H7*Precios!$B$10</f>
+        <f>H6*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K7" s="7">
-        <f>I7*Precios!$B$10</f>
+        <f>I6*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L7" s="7">
-        <f>(D7*E7*Precios!$C$4+F7*Precios!$C$5+G7*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D6*E6*Precios!$C$4+F6*Precios!$C$5+G6*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M7" s="6">
-        <f>K7*Precios!$B$11</f>
+        <f>K6*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N7" s="7">
-        <f>I7*Precios!$B$13</f>
+        <f>I6*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O7" s="7">
-        <f>K7*Precios!$B$13</f>
+        <f>K6*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P7" s="7">
-        <f>K7*Precios!$B$14</f>
+        <f>K6*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1009,60 +956,60 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>~30 anuncios, 3 meses</t>
+          <t>hasta 10 anuncios, 1 mes</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>976</v>
+        <v>569</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>85</v>
+        <v>46</v>
       </c>
       <c r="H8" s="6">
-        <f>(D8*E8+F8+G8)*1000</f>
+        <f>(D7*E7+F7+G7)*1000</f>
         <v/>
       </c>
       <c r="I8" s="7">
-        <f>(D8*E8*Precios!$B$4+F8*Precios!$B$5+G8*Precios!$B$6)/1000</f>
+        <f>(D7*E7*Precios!$B$4+F7*Precios!$B$5+G7*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J8" s="6">
-        <f>H8*Precios!$B$10</f>
+        <f>H7*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K8" s="7">
-        <f>I8*Precios!$B$10</f>
+        <f>I7*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L8" s="7">
-        <f>(D8*E8*Precios!$C$4+F8*Precios!$C$5+G8*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D7*E7*Precios!$C$4+F7*Precios!$C$5+G7*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M8" s="6">
-        <f>K8*Precios!$B$11</f>
+        <f>K7*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N8" s="7">
-        <f>I8*Precios!$B$13</f>
+        <f>I7*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O8" s="7">
-        <f>K8*Precios!$B$13</f>
+        <f>K7*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P8" s="7">
-        <f>K8*Precios!$B$14</f>
+        <f>K7*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1074,125 +1021,125 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>100+ anuncios, 12 meses con desglose diario</t>
+          <t>~30 anuncios, 3 meses</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>144</v>
+        <v>116</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>2095</v>
+        <v>976</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>184</v>
+        <v>85</v>
       </c>
       <c r="H9" s="6">
-        <f>(D9*E9+F9+G9)*1000</f>
+        <f>(D8*E8+F8+G8)*1000</f>
         <v/>
       </c>
       <c r="I9" s="7">
-        <f>(D9*E9*Precios!$B$4+F9*Precios!$B$5+G9*Precios!$B$6)/1000</f>
+        <f>(D8*E8*Precios!$B$4+F8*Precios!$B$5+G8*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J9" s="6">
-        <f>H9*Precios!$B$10</f>
+        <f>H8*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K9" s="7">
-        <f>I9*Precios!$B$10</f>
+        <f>I8*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L9" s="7">
-        <f>(D9*E9*Precios!$C$4+F9*Precios!$C$5+G9*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D8*E8*Precios!$C$4+F8*Precios!$C$5+G8*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M9" s="6">
-        <f>K9*Precios!$B$11</f>
+        <f>K8*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N9" s="7">
-        <f>I9*Precios!$B$13</f>
+        <f>I8*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O9" s="7">
-        <f>K9*Precios!$B$13</f>
+        <f>K8*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P9" s="7">
-        <f>K9*Precios!$B$14</f>
+        <f>K8*Precios!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>Meta Ads</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>hasta 5 campañas, sin términos de búsqueda</t>
+          <t>100+ anuncios, 12 meses con desglose diario</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>569</v>
+        <v>2095</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>46</v>
+        <v>184</v>
       </c>
       <c r="H10" s="6">
-        <f>(D10*E10+F10+G10)*1000</f>
+        <f>(D9*E9+F9+G9)*1000</f>
         <v/>
       </c>
       <c r="I10" s="7">
-        <f>(D10*E10*Precios!$B$4+F10*Precios!$B$5+G10*Precios!$B$6)/1000</f>
+        <f>(D9*E9*Precios!$B$4+F9*Precios!$B$5+G9*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J10" s="6">
-        <f>H10*Precios!$B$10</f>
+        <f>H9*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K10" s="7">
-        <f>I10*Precios!$B$10</f>
+        <f>I9*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L10" s="7">
-        <f>(D10*E10*Precios!$C$4+F10*Precios!$C$5+G10*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D9*E9*Precios!$C$4+F9*Precios!$C$5+G9*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M10" s="6">
-        <f>K10*Precios!$B$11</f>
+        <f>K9*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N10" s="7">
-        <f>I10*Precios!$B$13</f>
+        <f>I9*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O10" s="7">
-        <f>K10*Precios!$B$13</f>
+        <f>K9*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P10" s="7">
-        <f>K10*Precios!$B$14</f>
+        <f>K9*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1204,60 +1151,60 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>~15 campañas con palabras clave</t>
+          <t>hasta 5 campañas, sin términos de búsqueda</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1046</v>
+        <v>569</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>85</v>
+        <v>46</v>
       </c>
       <c r="H11" s="6">
-        <f>(D11*E11+F11+G11)*1000</f>
+        <f>(D10*E10+F10+G10)*1000</f>
         <v/>
       </c>
       <c r="I11" s="7">
-        <f>(D11*E11*Precios!$B$4+F11*Precios!$B$5+G11*Precios!$B$6)/1000</f>
+        <f>(D10*E10*Precios!$B$4+F10*Precios!$B$5+G10*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J11" s="6">
-        <f>H11*Precios!$B$10</f>
+        <f>H10*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K11" s="7">
-        <f>I11*Precios!$B$10</f>
+        <f>I10*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L11" s="7">
-        <f>(D11*E11*Precios!$C$4+F11*Precios!$C$5+G11*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D10*E10*Precios!$C$4+F10*Precios!$C$5+G10*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M11" s="6">
-        <f>K11*Precios!$B$11</f>
+        <f>K10*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N11" s="7">
-        <f>I11*Precios!$B$13</f>
+        <f>I10*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O11" s="7">
-        <f>K11*Precios!$B$13</f>
+        <f>K10*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P11" s="7">
-        <f>K11*Precios!$B$14</f>
+        <f>K10*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1269,125 +1216,125 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>50+ campañas con términos de búsqueda</t>
+          <t>~15 campañas con palabras clave</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>150</v>
+        <v>121</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>2205</v>
+        <v>1046</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>184</v>
+        <v>85</v>
       </c>
       <c r="H12" s="6">
-        <f>(D12*E12+F12+G12)*1000</f>
+        <f>(D11*E11+F11+G11)*1000</f>
         <v/>
       </c>
       <c r="I12" s="7">
-        <f>(D12*E12*Precios!$B$4+F12*Precios!$B$5+G12*Precios!$B$6)/1000</f>
+        <f>(D11*E11*Precios!$B$4+F11*Precios!$B$5+G11*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J12" s="6">
-        <f>H12*Precios!$B$10</f>
+        <f>H11*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K12" s="7">
-        <f>I12*Precios!$B$10</f>
+        <f>I11*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L12" s="7">
-        <f>(D12*E12*Precios!$C$4+F12*Precios!$C$5+G12*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D11*E11*Precios!$C$4+F11*Precios!$C$5+G11*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M12" s="6">
-        <f>K12*Precios!$B$11</f>
+        <f>K11*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N12" s="7">
-        <f>I12*Precios!$B$13</f>
+        <f>I11*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O12" s="7">
-        <f>K12*Precios!$B$13</f>
+        <f>K11*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P12" s="7">
-        <f>K12*Precios!$B$14</f>
+        <f>K11*Precios!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LinkedIn Ads</t>
+          <t>Google Ads</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1 a 3 campañas</t>
+          <t>50+ campañas con términos de búsqueda</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>466</v>
+        <v>2205</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>40</v>
+        <v>184</v>
       </c>
       <c r="H13" s="6">
-        <f>(D13*E13+F13+G13)*1000</f>
+        <f>(D12*E12+F12+G12)*1000</f>
         <v/>
       </c>
       <c r="I13" s="7">
-        <f>(D13*E13*Precios!$B$4+F13*Precios!$B$5+G13*Precios!$B$6)/1000</f>
+        <f>(D12*E12*Precios!$B$4+F12*Precios!$B$5+G12*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J13" s="6">
-        <f>H13*Precios!$B$10</f>
+        <f>H12*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K13" s="7">
-        <f>I13*Precios!$B$10</f>
+        <f>I12*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L13" s="7">
-        <f>(D13*E13*Precios!$C$4+F13*Precios!$C$5+G13*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D12*E12*Precios!$C$4+F12*Precios!$C$5+G12*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M13" s="6">
-        <f>K13*Precios!$B$11</f>
+        <f>K12*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N13" s="7">
-        <f>I13*Precios!$B$13</f>
+        <f>I12*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O13" s="7">
-        <f>K13*Precios!$B$13</f>
+        <f>K12*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P13" s="7">
-        <f>K13*Precios!$B$14</f>
+        <f>K12*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1399,60 +1346,60 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>~10 campañas</t>
+          <t>1 a 3 campañas</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>803</v>
+        <v>466</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H14" s="6">
-        <f>(D14*E14+F14+G14)*1000</f>
+        <f>(D13*E13+F13+G13)*1000</f>
         <v/>
       </c>
       <c r="I14" s="7">
-        <f>(D14*E14*Precios!$B$4+F14*Precios!$B$5+G14*Precios!$B$6)/1000</f>
+        <f>(D13*E13*Precios!$B$4+F13*Precios!$B$5+G13*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J14" s="6">
-        <f>H14*Precios!$B$10</f>
+        <f>H13*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K14" s="7">
-        <f>I14*Precios!$B$10</f>
+        <f>I13*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L14" s="7">
-        <f>(D14*E14*Precios!$C$4+F14*Precios!$C$5+G14*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D13*E13*Precios!$C$4+F13*Precios!$C$5+G13*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M14" s="6">
-        <f>K14*Precios!$B$11</f>
+        <f>K13*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N14" s="7">
-        <f>I14*Precios!$B$13</f>
+        <f>I13*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O14" s="7">
-        <f>K14*Precios!$B$13</f>
+        <f>K13*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P14" s="7">
-        <f>K14*Precios!$B$14</f>
+        <f>K13*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1464,125 +1411,125 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>30+ campañas con datos demográficos</t>
+          <t>~10 campañas</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>1654</v>
+        <v>803</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>147</v>
+        <v>70</v>
       </c>
       <c r="H15" s="6">
-        <f>(D15*E15+F15+G15)*1000</f>
+        <f>(D14*E14+F14+G14)*1000</f>
         <v/>
       </c>
       <c r="I15" s="7">
-        <f>(D15*E15*Precios!$B$4+F15*Precios!$B$5+G15*Precios!$B$6)/1000</f>
+        <f>(D14*E14*Precios!$B$4+F14*Precios!$B$5+G14*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J15" s="6">
-        <f>H15*Precios!$B$10</f>
+        <f>H14*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K15" s="7">
-        <f>I15*Precios!$B$10</f>
+        <f>I14*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L15" s="7">
-        <f>(D15*E15*Precios!$C$4+F15*Precios!$C$5+G15*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D14*E14*Precios!$C$4+F14*Precios!$C$5+G14*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M15" s="6">
-        <f>K15*Precios!$B$11</f>
+        <f>K14*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N15" s="7">
-        <f>I15*Precios!$B$13</f>
+        <f>I14*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O15" s="7">
-        <f>K15*Precios!$B$13</f>
+        <f>K14*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P15" s="7">
-        <f>K15*Precios!$B$14</f>
+        <f>K14*Precios!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WhatsApp Marketing</t>
+          <t>LinkedIn Ads</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1 o 2 envíos masivos</t>
+          <t>30+ campañas con datos demográficos</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>466</v>
+        <v>1654</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="H16" s="6">
-        <f>(D16*E16+F16+G16)*1000</f>
+        <f>(D15*E15+F15+G15)*1000</f>
         <v/>
       </c>
       <c r="I16" s="7">
-        <f>(D16*E16*Precios!$B$4+F16*Precios!$B$5+G16*Precios!$B$6)/1000</f>
+        <f>(D15*E15*Precios!$B$4+F15*Precios!$B$5+G15*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J16" s="6">
-        <f>H16*Precios!$B$10</f>
+        <f>H15*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K16" s="7">
-        <f>I16*Precios!$B$10</f>
+        <f>I15*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L16" s="7">
-        <f>(D16*E16*Precios!$C$4+F16*Precios!$C$5+G16*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D15*E15*Precios!$C$4+F15*Precios!$C$5+G15*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M16" s="6">
-        <f>K16*Precios!$B$11</f>
+        <f>K15*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N16" s="7">
-        <f>I16*Precios!$B$13</f>
+        <f>I15*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O16" s="7">
-        <f>K16*Precios!$B$13</f>
+        <f>K15*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P16" s="7">
-        <f>K16*Precios!$B$14</f>
+        <f>K15*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1594,60 +1541,60 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>~6 envíos</t>
+          <t>1 o 2 envíos masivos</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>767</v>
+        <v>466</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H17" s="6">
-        <f>(D17*E17+F17+G17)*1000</f>
+        <f>(D16*E16+F16+G16)*1000</f>
         <v/>
       </c>
       <c r="I17" s="7">
-        <f>(D17*E17*Precios!$B$4+F17*Precios!$B$5+G17*Precios!$B$6)/1000</f>
+        <f>(D16*E16*Precios!$B$4+F16*Precios!$B$5+G16*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J17" s="6">
-        <f>H17*Precios!$B$10</f>
+        <f>H16*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K17" s="7">
-        <f>I17*Precios!$B$10</f>
+        <f>I16*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L17" s="7">
-        <f>(D17*E17*Precios!$C$4+F17*Precios!$C$5+G17*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D16*E16*Precios!$C$4+F16*Precios!$C$5+G16*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M17" s="6">
-        <f>K17*Precios!$B$11</f>
+        <f>K16*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N17" s="7">
-        <f>I17*Precios!$B$13</f>
+        <f>I16*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O17" s="7">
-        <f>K17*Precios!$B$13</f>
+        <f>K16*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P17" s="7">
-        <f>K17*Precios!$B$14</f>
+        <f>K16*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1659,125 +1606,125 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>20+ envíos con plantillas y respuestas</t>
+          <t>~6 envíos</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>1597</v>
+        <v>767</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>147</v>
+        <v>70</v>
       </c>
       <c r="H18" s="6">
-        <f>(D18*E18+F18+G18)*1000</f>
+        <f>(D17*E17+F17+G17)*1000</f>
         <v/>
       </c>
       <c r="I18" s="7">
-        <f>(D18*E18*Precios!$B$4+F18*Precios!$B$5+G18*Precios!$B$6)/1000</f>
+        <f>(D17*E17*Precios!$B$4+F17*Precios!$B$5+G17*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J18" s="6">
-        <f>H18*Precios!$B$10</f>
+        <f>H17*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>I18*Precios!$B$10</f>
+        <f>I17*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L18" s="7">
-        <f>(D18*E18*Precios!$C$4+F18*Precios!$C$5+G18*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D17*E17*Precios!$C$4+F17*Precios!$C$5+G17*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M18" s="6">
-        <f>K18*Precios!$B$11</f>
+        <f>K17*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N18" s="7">
-        <f>I18*Precios!$B$13</f>
+        <f>I17*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O18" s="7">
-        <f>K18*Precios!$B$13</f>
+        <f>K17*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P18" s="7">
-        <f>K18*Precios!$B$14</f>
+        <f>K17*Precios!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Email Marketing</t>
+          <t>WhatsApp Marketing</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1 a 3 campañas</t>
+          <t>20+ envíos con plantillas y respuestas</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>466</v>
+        <v>1597</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="H19" s="6">
-        <f>(D19*E19+F19+G19)*1000</f>
+        <f>(D18*E18+F18+G18)*1000</f>
         <v/>
       </c>
       <c r="I19" s="7">
-        <f>(D19*E19*Precios!$B$4+F19*Precios!$B$5+G19*Precios!$B$6)/1000</f>
+        <f>(D18*E18*Precios!$B$4+F18*Precios!$B$5+G18*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J19" s="6">
-        <f>H19*Precios!$B$10</f>
+        <f>H18*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K19" s="7">
-        <f>I19*Precios!$B$10</f>
+        <f>I18*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L19" s="7">
-        <f>(D19*E19*Precios!$C$4+F19*Precios!$C$5+G19*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D18*E18*Precios!$C$4+F18*Precios!$C$5+G18*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M19" s="6">
-        <f>K19*Precios!$B$11</f>
+        <f>K18*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N19" s="7">
-        <f>I19*Precios!$B$13</f>
+        <f>I18*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O19" s="7">
-        <f>K19*Precios!$B$13</f>
+        <f>K18*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P19" s="7">
-        <f>K19*Precios!$B$14</f>
+        <f>K18*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1789,60 +1736,60 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>~10 campañas</t>
+          <t>1 a 3 campañas</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>803</v>
+        <v>466</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H20" s="6">
-        <f>(D20*E20+F20+G20)*1000</f>
+        <f>(D19*E19+F19+G19)*1000</f>
         <v/>
       </c>
       <c r="I20" s="7">
-        <f>(D20*E20*Precios!$B$4+F20*Precios!$B$5+G20*Precios!$B$6)/1000</f>
+        <f>(D19*E19*Precios!$B$4+F19*Precios!$B$5+G19*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J20" s="6">
-        <f>H20*Precios!$B$10</f>
+        <f>H19*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>I20*Precios!$B$10</f>
+        <f>I19*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L20" s="7">
-        <f>(D20*E20*Precios!$C$4+F20*Precios!$C$5+G20*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D19*E19*Precios!$C$4+F19*Precios!$C$5+G19*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M20" s="6">
-        <f>K20*Precios!$B$11</f>
+        <f>K19*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N20" s="7">
-        <f>I20*Precios!$B$13</f>
+        <f>I19*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O20" s="7">
-        <f>K20*Precios!$B$13</f>
+        <f>K19*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P20" s="7">
-        <f>K20*Precios!$B$14</f>
+        <f>K19*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1854,125 +1801,125 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>30+ campañas y flujos automáticos</t>
+          <t>~10 campañas</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>1654</v>
+        <v>803</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>147</v>
+        <v>70</v>
       </c>
       <c r="H21" s="6">
-        <f>(D21*E21+F21+G21)*1000</f>
+        <f>(D20*E20+F20+G20)*1000</f>
         <v/>
       </c>
       <c r="I21" s="7">
-        <f>(D21*E21*Precios!$B$4+F21*Precios!$B$5+G21*Precios!$B$6)/1000</f>
+        <f>(D20*E20*Precios!$B$4+F20*Precios!$B$5+G20*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J21" s="6">
-        <f>H21*Precios!$B$10</f>
+        <f>H20*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K21" s="7">
-        <f>I21*Precios!$B$10</f>
+        <f>I20*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L21" s="7">
-        <f>(D21*E21*Precios!$C$4+F21*Precios!$C$5+G21*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D20*E20*Precios!$C$4+F20*Precios!$C$5+G20*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M21" s="6">
-        <f>K21*Precios!$B$11</f>
+        <f>K20*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N21" s="7">
-        <f>I21*Precios!$B$13</f>
+        <f>I20*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O21" s="7">
-        <f>K21*Precios!$B$13</f>
+        <f>K20*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P21" s="7">
-        <f>K21*Precios!$B$14</f>
+        <f>K20*Precios!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cruce omnicanal</t>
+          <t>Email Marketing</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2 o 3 canales</t>
+          <t>30+ campañas y flujos automáticos</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>518</v>
+        <v>1654</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>46</v>
+        <v>147</v>
       </c>
       <c r="H22" s="6">
-        <f>(D22*E22+F22+G22)*1000</f>
+        <f>(D21*E21+F21+G21)*1000</f>
         <v/>
       </c>
       <c r="I22" s="7">
-        <f>(D22*E22*Precios!$B$4+F22*Precios!$B$5+G22*Precios!$B$6)/1000</f>
+        <f>(D21*E21*Precios!$B$4+F21*Precios!$B$5+G21*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J22" s="6">
-        <f>H22*Precios!$B$10</f>
+        <f>H21*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>I22*Precios!$B$10</f>
+        <f>I21*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L22" s="7">
-        <f>(D22*E22*Precios!$C$4+F22*Precios!$C$5+G22*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D21*E21*Precios!$C$4+F21*Precios!$C$5+G21*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M22" s="6">
-        <f>K22*Precios!$B$11</f>
+        <f>K21*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N22" s="7">
-        <f>I22*Precios!$B$13</f>
+        <f>I21*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O22" s="7">
-        <f>K22*Precios!$B$13</f>
+        <f>K21*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P22" s="7">
-        <f>K22*Precios!$B$14</f>
+        <f>K21*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -1984,60 +1931,60 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4 o 5 canales</t>
+          <t>2 o 3 canales</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>1046</v>
+        <v>518</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="H23" s="6">
-        <f>(D23*E23+F23+G23)*1000</f>
+        <f>(D22*E22+F22+G22)*1000</f>
         <v/>
       </c>
       <c r="I23" s="7">
-        <f>(D23*E23*Precios!$B$4+F23*Precios!$B$5+G23*Precios!$B$6)/1000</f>
+        <f>(D22*E22*Precios!$B$4+F22*Precios!$B$5+G22*Precios!$B$6)/1000</f>
         <v/>
       </c>
       <c r="J23" s="6">
-        <f>H23*Precios!$B$10</f>
+        <f>H22*Precios!$B$10</f>
         <v/>
       </c>
       <c r="K23" s="7">
-        <f>I23*Precios!$B$10</f>
+        <f>I22*Precios!$B$10</f>
         <v/>
       </c>
       <c r="L23" s="7">
-        <f>(D23*E23*Precios!$C$4+F23*Precios!$C$5+G23*Precios!$C$6)/1000*Precios!$B$10</f>
+        <f>(D22*E22*Precios!$C$4+F22*Precios!$C$5+G22*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
       <c r="M23" s="6">
-        <f>K23*Precios!$B$11</f>
+        <f>K22*Precios!$B$11</f>
         <v/>
       </c>
       <c r="N23" s="7">
-        <f>I23*Precios!$B$13</f>
+        <f>I22*Precios!$B$13</f>
         <v/>
       </c>
       <c r="O23" s="7">
-        <f>K23*Precios!$B$13</f>
+        <f>K22*Precios!$B$13</f>
         <v/>
       </c>
       <c r="P23" s="7">
-        <f>K23*Precios!$B$14</f>
+        <f>K22*Precios!$B$14</f>
         <v/>
       </c>
     </row>
@@ -2049,188 +1996,254 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>4 o 5 canales</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>178</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>1046</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="H24" s="6">
+        <f>(D23*E23+F23+G23)*1000</f>
+        <v/>
+      </c>
+      <c r="I24" s="7">
+        <f>(D23*E23*Precios!$B$4+F23*Precios!$B$5+G23*Precios!$B$6)/1000</f>
+        <v/>
+      </c>
+      <c r="J24" s="6">
+        <f>H23*Precios!$B$10</f>
+        <v/>
+      </c>
+      <c r="K24" s="7">
+        <f>I23*Precios!$B$10</f>
+        <v/>
+      </c>
+      <c r="L24" s="7">
+        <f>(D23*E23*Precios!$C$4+F23*Precios!$C$5+G23*Precios!$C$6)/1000*Precios!$B$10</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>K23*Precios!$B$11</f>
+        <v/>
+      </c>
+      <c r="N24" s="7">
+        <f>I23*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="O24" s="7">
+        <f>K23*Precios!$B$13</f>
+        <v/>
+      </c>
+      <c r="P24" s="7">
+        <f>K23*Precios!$B$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cruce omnicanal</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>Grande</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>6 canales con atribución cruzada</t>
         </is>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D25" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E25" s="5" t="n">
         <v>230</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F25" s="5" t="n">
         <v>2205</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="G25" s="5" t="n">
         <v>196</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H25" s="6">
         <f>(D24*E24+F24+G24)*1000</f>
         <v/>
       </c>
-      <c r="I24" s="7">
+      <c r="I25" s="7">
         <f>(D24*E24*Precios!$B$4+F24*Precios!$B$5+G24*Precios!$B$6)/1000</f>
         <v/>
       </c>
-      <c r="J24" s="6">
+      <c r="J25" s="6">
         <f>H24*Precios!$B$10</f>
         <v/>
       </c>
-      <c r="K24" s="7">
+      <c r="K25" s="7">
         <f>I24*Precios!$B$10</f>
         <v/>
       </c>
-      <c r="L24" s="7">
+      <c r="L25" s="7">
         <f>(D24*E24*Precios!$C$4+F24*Precios!$C$5+G24*Precios!$C$6)/1000*Precios!$B$10</f>
         <v/>
       </c>
-      <c r="M24" s="6">
+      <c r="M25" s="6">
         <f>K24*Precios!$B$11</f>
         <v/>
       </c>
-      <c r="N24" s="7">
+      <c r="N25" s="7">
         <f>I24*Precios!$B$13</f>
         <v/>
       </c>
-      <c r="O24" s="7">
+      <c r="O25" s="7">
         <f>K24*Precios!$B$13</f>
         <v/>
       </c>
-      <c r="P24" s="7">
+      <c r="P25" s="7">
         <f>K24*Precios!$B$14</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>Tablero omnicanal completo · Chica</t>
-        </is>
-      </c>
-      <c r="H26" s="8">
-        <f>SUMIF($B$4:$B$24,"Chica",H$4:H$24)</f>
-        <v/>
-      </c>
-      <c r="I26" s="9">
-        <f>SUMIF($B$4:$B$24,"Chica",I$4:I$24)</f>
-        <v/>
-      </c>
-      <c r="J26" s="8">
-        <f>SUMIF($B$4:$B$24,"Chica",J$4:J$24)</f>
-        <v/>
-      </c>
-      <c r="K26" s="9">
-        <f>SUMIF($B$4:$B$24,"Chica",K$4:K$24)</f>
-        <v/>
-      </c>
-      <c r="L26" s="9">
-        <f>SUMIF($B$4:$B$24,"Chica",L$4:L$24)</f>
-        <v/>
-      </c>
-      <c r="M26" s="8">
-        <f>SUMIF($B$4:$B$24,"Chica",M$4:M$24)</f>
-        <v/>
-      </c>
-      <c r="N26">
-        <f>SUMIF($B$4:$B$24,"Chica",N$4:N$24)</f>
-        <v/>
-      </c>
-      <c r="O26">
-        <f>SUMIF($B$4:$B$24,"Chica",O$4:O$24)</f>
-        <v/>
-      </c>
-      <c r="P26">
-        <f>SUMIF($B$4:$B$24,"Chica",P$4:P$24)</f>
-        <v/>
-      </c>
-    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Tablero omnicanal completo · Mediana</t>
+          <t>Tablero omnicanal completo · Chica</t>
         </is>
       </c>
       <c r="H27" s="8">
-        <f>SUMIF($B$4:$B$24,"Mediana",H$4:H$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",H$4:H$24)</f>
         <v/>
       </c>
       <c r="I27" s="9">
-        <f>SUMIF($B$4:$B$24,"Mediana",I$4:I$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",I$4:I$24)</f>
         <v/>
       </c>
       <c r="J27" s="8">
-        <f>SUMIF($B$4:$B$24,"Mediana",J$4:J$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",J$4:J$24)</f>
         <v/>
       </c>
       <c r="K27" s="9">
-        <f>SUMIF($B$4:$B$24,"Mediana",K$4:K$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",K$4:K$24)</f>
         <v/>
       </c>
       <c r="L27" s="9">
-        <f>SUMIF($B$4:$B$24,"Mediana",L$4:L$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",L$4:L$24)</f>
         <v/>
       </c>
       <c r="M27" s="8">
-        <f>SUMIF($B$4:$B$24,"Mediana",M$4:M$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",M$4:M$24)</f>
         <v/>
       </c>
       <c r="N27">
-        <f>SUMIF($B$4:$B$24,"Mediana",N$4:N$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",N$4:N$24)</f>
         <v/>
       </c>
       <c r="O27">
-        <f>SUMIF($B$4:$B$24,"Mediana",O$4:O$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",O$4:O$24)</f>
         <v/>
       </c>
       <c r="P27">
-        <f>SUMIF($B$4:$B$24,"Mediana",P$4:P$24)</f>
+        <f>SUMIF($B$4:$B$24,"Chica",P$4:P$24)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
+          <t>Tablero omnicanal completo · Mediana</t>
+        </is>
+      </c>
+      <c r="H28" s="8">
+        <f>SUMIF($B$4:$B$24,"Mediana",H$4:H$24)</f>
+        <v/>
+      </c>
+      <c r="I28" s="9">
+        <f>SUMIF($B$4:$B$24,"Mediana",I$4:I$24)</f>
+        <v/>
+      </c>
+      <c r="J28" s="8">
+        <f>SUMIF($B$4:$B$24,"Mediana",J$4:J$24)</f>
+        <v/>
+      </c>
+      <c r="K28" s="9">
+        <f>SUMIF($B$4:$B$24,"Mediana",K$4:K$24)</f>
+        <v/>
+      </c>
+      <c r="L28" s="9">
+        <f>SUMIF($B$4:$B$24,"Mediana",L$4:L$24)</f>
+        <v/>
+      </c>
+      <c r="M28" s="8">
+        <f>SUMIF($B$4:$B$24,"Mediana",M$4:M$24)</f>
+        <v/>
+      </c>
+      <c r="N28">
+        <f>SUMIF($B$4:$B$24,"Mediana",N$4:N$24)</f>
+        <v/>
+      </c>
+      <c r="O28">
+        <f>SUMIF($B$4:$B$24,"Mediana",O$4:O$24)</f>
+        <v/>
+      </c>
+      <c r="P28">
+        <f>SUMIF($B$4:$B$24,"Mediana",P$4:P$24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
           <t>Tablero omnicanal completo · Grande</t>
         </is>
       </c>
-      <c r="H28" s="8">
+      <c r="H29" s="8">
         <f>SUMIF($B$4:$B$24,"Grande",H$4:H$24)</f>
         <v/>
       </c>
-      <c r="I28" s="9">
+      <c r="I29" s="9">
         <f>SUMIF($B$4:$B$24,"Grande",I$4:I$24)</f>
         <v/>
       </c>
-      <c r="J28" s="8">
+      <c r="J29" s="8">
         <f>SUMIF($B$4:$B$24,"Grande",J$4:J$24)</f>
         <v/>
       </c>
-      <c r="K28" s="9">
+      <c r="K29" s="9">
         <f>SUMIF($B$4:$B$24,"Grande",K$4:K$24)</f>
         <v/>
       </c>
-      <c r="L28" s="9">
+      <c r="L29" s="9">
         <f>SUMIF($B$4:$B$24,"Grande",L$4:L$24)</f>
         <v/>
       </c>
-      <c r="M28" s="8">
+      <c r="M29" s="8">
         <f>SUMIF($B$4:$B$24,"Grande",M$4:M$24)</f>
         <v/>
       </c>
-      <c r="N28">
+      <c r="N29">
         <f>SUMIF($B$4:$B$24,"Grande",N$4:N$24)</f>
         <v/>
       </c>
-      <c r="O28">
+      <c r="O29">
         <f>SUMIF($B$4:$B$24,"Grande",O$4:O$24)</f>
         <v/>
       </c>
-      <c r="P28">
+      <c r="P29">
         <f>SUMIF($B$4:$B$24,"Grande",P$4:P$24)</f>
         <v/>
       </c>
@@ -2748,7 +2761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2762,89 +2775,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>DESACTUALIZADO: estos valores se calibraron con costos inflados por la conversación larga. La versión vigente es AUREA_Costo_IC.html (costos en sesión nueva, medidos llamada por llamada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Costo por actualización (USD, Opus 5.5) aplicando mejoras que no sacrifican calidad</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Paso 1: sesión nueva por export, sin compactación, y verificación con el verificador automático + 2 capturas (contexto nuevo escrito −36%). Paso 2: además, una sola sesión por cliente con todos los canales (caché compartido, −30%). Paso 3: además, pipeline propio por API con caché de 5 minutos (escritura USD 5 en vez de 8).</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Canal</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Tamaño</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Hoy (cuadro)</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Paso 1</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Paso 2</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>Paso 3</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Precio 2,5x sobre Paso 2</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Precio 4x sobre Paso 2</t>
         </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Prometheo (CRM)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Chica</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>1.89</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>4.73</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>7.56</v>
       </c>
     </row>
     <row r="6">
@@ -2855,26 +2846,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>6.88</v>
+        <v>3.71</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>5.08</v>
+        <v>2.7</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3.55</v>
+        <v>1.89</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>2.71</v>
+        <v>1.42</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>8.880000000000001</v>
+        <v>4.73</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>14.21</v>
+        <v>7.56</v>
       </c>
     </row>
     <row r="7">
@@ -2885,56 +2876,56 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>14.71</v>
+        <v>6.88</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>10.78</v>
+        <v>5.08</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7.55</v>
+        <v>3.55</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>5.71</v>
+        <v>2.71</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>18.87</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>30.18</v>
+        <v>14.21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Meta Ads</t>
+          <t>Prometheo (CRM)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2.69</v>
+        <v>14.71</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>1.95</v>
+        <v>10.78</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>1.36</v>
+        <v>7.55</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1.02</v>
+        <v>5.71</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>3.41</v>
+        <v>18.87</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>5.46</v>
+        <v>30.18</v>
       </c>
     </row>
     <row r="9">
@@ -2945,26 +2936,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>4.64</v>
+        <v>2.69</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>3.38</v>
+        <v>1.95</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2.37</v>
+        <v>1.36</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.78</v>
+        <v>1.02</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>5.91</v>
+        <v>3.41</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>9.460000000000001</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="10">
@@ -2975,56 +2966,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>9.92</v>
+        <v>4.64</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>7.21</v>
+        <v>3.38</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>5.05</v>
+        <v>2.37</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>3.78</v>
+        <v>1.78</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>12.62</v>
+        <v>5.91</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>20.18</v>
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>Meta Ads</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>2.69</v>
+        <v>9.92</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>1.95</v>
+        <v>7.21</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1.36</v>
+        <v>5.05</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1.02</v>
+        <v>3.78</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>3.41</v>
+        <v>12.62</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>5.46</v>
+        <v>20.18</v>
       </c>
     </row>
     <row r="12">
@@ -3035,26 +3026,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>4.94</v>
+        <v>2.69</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>3.59</v>
+        <v>1.95</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2.51</v>
+        <v>1.36</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1.88</v>
+        <v>1.02</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>6.28</v>
+        <v>3.41</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10.05</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="13">
@@ -3065,56 +3056,56 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>10.4</v>
+        <v>4.94</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>7.55</v>
+        <v>3.59</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>5.28</v>
+        <v>2.51</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>3.95</v>
+        <v>1.88</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>13.21</v>
+        <v>6.28</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>21.13</v>
+        <v>10.05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LinkedIn Ads</t>
+          <t>Google Ads</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>2.21</v>
+        <v>10.4</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1.6</v>
+        <v>7.55</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>1.12</v>
+        <v>5.28</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.84</v>
+        <v>3.95</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>2.81</v>
+        <v>13.21</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>4.49</v>
+        <v>21.13</v>
       </c>
     </row>
     <row r="15">
@@ -3125,26 +3116,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>3.81</v>
+        <v>2.21</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2.77</v>
+        <v>1.6</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1.94</v>
+        <v>1.12</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1.45</v>
+        <v>0.84</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>4.84</v>
+        <v>2.81</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>7.75</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="16">
@@ -3155,56 +3146,56 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>7.8</v>
+        <v>3.81</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>5.66</v>
+        <v>2.77</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>3.96</v>
+        <v>1.94</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2.96</v>
+        <v>1.45</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>9.9</v>
+        <v>4.84</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>15.84</v>
+        <v>7.75</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WhatsApp Marketing</t>
+          <t>LinkedIn Ads</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>2.21</v>
+        <v>7.8</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>1.6</v>
+        <v>5.66</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1.12</v>
+        <v>3.96</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>0.84</v>
+        <v>2.96</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>2.81</v>
+        <v>9.9</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>4.49</v>
+        <v>15.84</v>
       </c>
     </row>
     <row r="18">
@@ -3215,26 +3206,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>3.68</v>
+        <v>2.21</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2.68</v>
+        <v>1.6</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>1.88</v>
+        <v>1.12</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>1.42</v>
+        <v>0.84</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.7</v>
+        <v>2.81</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>7.52</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="19">
@@ -3245,56 +3236,56 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>7.57</v>
+        <v>3.68</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>5.5</v>
+        <v>2.68</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>3.85</v>
+        <v>1.88</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>2.89</v>
+        <v>1.42</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>9.630000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>15.4</v>
+        <v>7.52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Email Marketing</t>
+          <t>WhatsApp Marketing</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>2.21</v>
+        <v>7.57</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>1.6</v>
+        <v>5.5</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>1.12</v>
+        <v>3.85</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>0.84</v>
+        <v>2.89</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>2.81</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>4.49</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="21">
@@ -3305,26 +3296,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>3.82</v>
+        <v>2.21</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>2.78</v>
+        <v>1.6</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>1.94</v>
+        <v>1.12</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>1.46</v>
+        <v>0.84</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>4.86</v>
+        <v>2.81</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>7.78</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="22">
@@ -3335,56 +3326,56 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Grande</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>7.81</v>
+        <v>3.82</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>5.67</v>
+        <v>2.78</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>3.97</v>
+        <v>1.94</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>2.97</v>
+        <v>1.46</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.92</v>
+        <v>4.86</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>15.87</v>
+        <v>7.78</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cruce omnicanal</t>
+          <t>Email Marketing</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Chica</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>2.53</v>
+        <v>7.81</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>1.86</v>
+        <v>5.67</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>1.3</v>
+        <v>3.97</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>0.99</v>
+        <v>2.97</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>3.25</v>
+        <v>9.92</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>5.21</v>
+        <v>15.87</v>
       </c>
     </row>
     <row r="24">
@@ -3395,26 +3386,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Chica</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>5.13</v>
+        <v>2.53</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>3.78</v>
+        <v>1.86</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>2.64</v>
+        <v>1.3</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>2.01</v>
+        <v>0.99</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>6.61</v>
+        <v>3.25</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>10.57</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="25">
@@ -3425,100 +3416,131 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>10.57</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cruce omnicanal</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>Grande</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C26" s="7" t="n">
         <v>10.74</v>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D26" s="7" t="n">
         <v>7.88</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="E26" s="7" t="n">
         <v>5.52</v>
       </c>
-      <c r="F25" s="7" t="n">
+      <c r="F26" s="7" t="n">
         <v>4.18</v>
       </c>
-      <c r="G25" s="7" t="n">
+      <c r="G26" s="7" t="n">
         <v>13.79</v>
       </c>
-      <c r="H25" s="7" t="n">
+      <c r="H26" s="7" t="n">
         <v>22.06</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Tablero completo · Chica</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="n">
-        <v>18.24</v>
-      </c>
-      <c r="D27" s="9" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="E27" s="9" t="n">
-        <v>9.289999999999999</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>6.98</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>23.23</v>
-      </c>
-      <c r="H27" s="9" t="n">
-        <v>37.17</v>
-      </c>
-    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>Tablero completo · Mediana</t>
+          <t>Tablero completo · Chica</t>
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>32.91</v>
+        <v>18.24</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>24.05</v>
+        <v>13.27</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>16.83</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>12.7</v>
+        <v>6.98</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>42.09</v>
+        <v>23.23</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>67.34</v>
+        <v>37.17</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
+          <t>Tablero completo · Mediana</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>32.91</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>24.05</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>16.83</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>67.34</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
           <t>Tablero completo · Grande</t>
         </is>
       </c>
-      <c r="C29" s="9" t="n">
+      <c r="C30" s="9" t="n">
         <v>68.95999999999999</v>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D30" s="9" t="n">
         <v>50.24</v>
       </c>
-      <c r="E29" s="9" t="n">
+      <c r="E30" s="9" t="n">
         <v>35.17</v>
       </c>
-      <c r="F29" s="9" t="n">
+      <c r="F30" s="9" t="n">
         <v>26.43</v>
       </c>
-      <c r="G29" s="9" t="n">
+      <c r="G30" s="9" t="n">
         <v>87.92</v>
       </c>
-      <c r="H29" s="9" t="n">
+      <c r="H30" s="9" t="n">
         <v>140.67</v>
       </c>
     </row>

</xml_diff>